<commit_message>
feat: add Essor favicon (app/icon) + apple-icon
</commit_message>
<xml_diff>
--- a/marketing/prospection/prospects-paysagistes.xlsx
+++ b/marketing/prospection/prospects-paysagistes.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -507,6 +507,11 @@
           <t>Statut</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Canal retenu</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -556,6 +561,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Formulaire</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -605,6 +615,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Formulaire</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -654,6 +669,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Formulaire</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -703,6 +723,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -752,6 +777,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Formulaire</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -799,6 +829,11 @@
       <c r="K7" s="2" t="inlineStr">
         <is>
           <t>À valider</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail)</t>
         </is>
       </c>
     </row>
@@ -846,6 +881,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -891,6 +931,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -938,6 +983,11 @@
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>À valider</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail)</t>
         </is>
       </c>
     </row>
@@ -985,6 +1035,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Formulaire</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1036,6 +1091,11 @@
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>À valider</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Formulaire + LinkedIn (suivre la page)</t>
         </is>
       </c>
     </row>
@@ -1083,6 +1143,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Formulaire</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1132,6 +1197,11 @@
           <t>À valider</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1183,6 +1253,11 @@
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>À valider</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Email (brouillon Gmail) + invitation LinkedIn</t>
         </is>
       </c>
     </row>

</xml_diff>